<commit_message>
New Features with Several bug fixes
</commit_message>
<xml_diff>
--- a/public/sample-products.xlsx
+++ b/public/sample-products.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20371"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\sme\public\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF548AD-97D8-47C1-BE06-DF4532F0AFD0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7230"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -25,27 +19,12 @@
     <t>name</t>
   </si>
   <si>
-    <t>basic_unit</t>
-  </si>
-  <si>
-    <t>buying_per_unit</t>
-  </si>
-  <si>
     <t>in_stock</t>
   </si>
   <si>
-    <t>retail_price_per_unit</t>
-  </si>
-  <si>
-    <t>wholesale_price_per_unit</t>
-  </si>
-  <si>
     <t>location</t>
   </si>
   <si>
-    <t>product_no</t>
-  </si>
-  <si>
     <t>barcode</t>
   </si>
   <si>
@@ -113,12 +92,27 @@
   </si>
   <si>
     <t>Test Product five</t>
+  </si>
+  <si>
+    <t>basic_uom</t>
+  </si>
+  <si>
+    <t>unit_cost</t>
+  </si>
+  <si>
+    <t>retail_price</t>
+  </si>
+  <si>
+    <t>wholesale_price</t>
+  </si>
+  <si>
+    <t>product_code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -665,7 +659,7 @@
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="Normal 2" xfId="42"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
     <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
@@ -829,37 +823,37 @@
     </dxf>
   </dxfs>
   <tableStyles count="8" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MAGADI-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="MAGADI-style" pivot="0" count="3">
       <tableStyleElement type="headerRow" dxfId="18"/>
       <tableStyleElement type="firstRowStripe" dxfId="17"/>
       <tableStyleElement type="secondRowStripe" dxfId="16"/>
     </tableStyle>
-    <tableStyle name="OSKT -style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
+    <tableStyle name="OSKT -style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="15"/>
       <tableStyleElement type="secondRowStripe" dxfId="14"/>
     </tableStyle>
-    <tableStyle name="OSSE-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
+    <tableStyle name="OSSE-style" pivot="0" count="3">
       <tableStyleElement type="headerRow" dxfId="13"/>
       <tableStyleElement type="firstRowStripe" dxfId="12"/>
       <tableStyleElement type="secondRowStripe" dxfId="11"/>
     </tableStyle>
-    <tableStyle name="OSMK-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
+    <tableStyle name="OSMK-style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="10"/>
       <tableStyleElement type="secondRowStripe" dxfId="9"/>
     </tableStyle>
-    <tableStyle name="OSTS-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
+    <tableStyle name="OSTS-style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="8"/>
       <tableStyleElement type="secondRowStripe" dxfId="7"/>
     </tableStyle>
-    <tableStyle name="LMKL-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF05000000}">
+    <tableStyle name="LMKL-style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="6"/>
       <tableStyleElement type="secondRowStripe" dxfId="5"/>
     </tableStyle>
-    <tableStyle name="TKTL-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF06000000}">
+    <tableStyle name="TKTL-style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="4"/>
       <tableStyleElement type="secondRowStripe" dxfId="3"/>
     </tableStyle>
-    <tableStyle name="ONML-style" pivot="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF07000000}">
+    <tableStyle name="ONML-style" pivot="0" count="2">
       <tableStyleElement type="firstRowStripe" dxfId="2"/>
       <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
@@ -918,7 +912,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -953,7 +947,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1130,24 +1124,24 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.90625" customWidth="1"/>
     <col min="3" max="3" width="42.26953125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.1796875" customWidth="1"/>
     <col min="8" max="8" width="22.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.453125" bestFit="1" customWidth="1"/>
@@ -1168,87 +1162,87 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
       <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" t="s">
+      <c r="S1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="T1" t="s">
         <v>12</v>
       </c>
-      <c r="P1" t="s">
+      <c r="U1" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="V1" t="s">
         <v>14</v>
       </c>
-      <c r="R1" t="s">
+      <c r="W1" t="s">
         <v>15</v>
-      </c>
-      <c r="S1" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" t="s">
-        <v>19</v>
-      </c>
-      <c r="W1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>76326532</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E2">
         <v>3600</v>
@@ -1265,16 +1259,16 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B3">
         <v>372882324</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>154</v>
@@ -1294,10 +1288,10 @@
         <v>87996545</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>256</v>
@@ -1317,10 +1311,10 @@
         <v>121323508</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E5">
         <v>302</v>
@@ -1337,10 +1331,10 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E6">
         <v>200</v>

</xml_diff>